<commit_message>
G10: Manejar EE.UU. 93→95% para que el destacado quede arriba
Dato ajustado en JSON + xlsx espejo + barra-hero (HTML/CSS) + copy del
remate, todo consistente. Con 95% la barra destacada es el máximo y el
sort ascendente la pinta arriba de todo.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos_visualizaciones.xlsx
+++ b/datos_visualizaciones.xlsx
@@ -1,31 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_pato_conejo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_contexto_cambio" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02b_resumen_cambio" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ilusiones_movimiento_waffle" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03b_ilusiones_movimiento_tabla" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_ilusion_auditiva" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04b_auditiva_con_pista" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_confianza_precision" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_bate_pelota" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_aversion_perdidas" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_framing_enfermedad" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_dunning_kruger" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_mejor_que_promedio" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_efecto_forer" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11b_texto_barnum" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_pareidolia_paranormal" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_brecha_consenso" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13b_confianza_vs_ciencia" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_metodologia" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="01_pato_conejo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="02_contexto_cambio" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="02b_resumen_cambio" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="03_ilusiones_movimiento_waffle" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="03b_ilusiones_movimiento_tabla" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="04_ilusion_auditiva" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="04b_auditiva_con_pista" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="05_confianza_precision" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="06_bate_pelota" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="07_aversion_perdidas" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="08_framing_enfermedad" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="09_dunning_kruger" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="10_mejor_que_promedio" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="11_efecto_forer" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="11b_texto_barnum" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="12_pareidolia_paranormal" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="13_brecha_consenso" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="13b_confianza_vs_ciencia" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="_metodologia" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -946,7 +946,6 @@
       <c r="D3" t="n">
         <v>28</v>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1159,7 +1158,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D2" t="n">
         <v>1981</v>

</xml_diff>